<commit_message>
refactor: use XmlSanitizer for document parsing
Replace raw XmlPullParser usage with XmlSanitizer across Excel and PowerPoint handlers to improve security and robustness when parsing untrusted document content.
</commit_message>
<xml_diff>
--- a/app/src/main/assets/samples/financial_model_q3.xlsx
+++ b/app/src/main/assets/samples/financial_model_q3.xlsx
@@ -8,9 +8,132 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
-<si><t>Category</t></si><si><t>Q1 Actual</t></si><si><t>Q2 Actual</t></si><si><t>Q3 Target</t></si><si><t>Variance %</t></si><si><t>Direct Enterprise Software</t></si><si><t>1,240,500</t></si><si><t>1,480,200</t></si><si><t>1,650,000</t></si><si><t>+11.4%</t></si><si><t>Cloud Infrastructure</t></si><si><t>340,000</t></si><si><t>365,000</t></si><si><t>380,000</t></si><si><t>+4.1%</t></si><si><t>Professional Services</t></si><si><t>190,000</t></si><si><t>210,000</t></si><si><t>230,000</t></si><si><t>+9.5%</t></si><si><t>Total Net Revenue</t></si><si><t>1,770,500</t></si><si><t>2,055,200</t></si><si><t>2,260,000</t></si><si><t>+10.0%</t></si><si><t>Department</t></si><si><t>Budget Allocation</t></si><si><t>Spent to Date</t></si><si><t>Remaining Balance</t></si><si><t>R&D Core Engineering</t></si><si><t>850,000</t></si><si><t>590,000</t></si><si><t>260,000</t></si><si><t>Product Design</t></si><si><t>220,000</t></si><si><t>145,000</t></si><si><t>75,000</t></si><si><t>Quality Assurance</t></si><si><t>160,000</t></si><si><t>110,000</t></si><si><t>50,000</t></si></sst>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Q1 Actual</t>
+  </si>
+  <si>
+    <t>Q2 Actual</t>
+  </si>
+  <si>
+    <t>Q3 Target</t>
+  </si>
+  <si>
+    <t>Variance %</t>
+  </si>
+  <si>
+    <t>Direct Enterprise Software</t>
+  </si>
+  <si>
+    <t>1,240,500</t>
+  </si>
+  <si>
+    <t>1,480,200</t>
+  </si>
+  <si>
+    <t>1,650,000</t>
+  </si>
+  <si>
+    <t>+11.4%</t>
+  </si>
+  <si>
+    <t>Cloud Infrastructure</t>
+  </si>
+  <si>
+    <t>340,000</t>
+  </si>
+  <si>
+    <t>365,000</t>
+  </si>
+  <si>
+    <t>380,000</t>
+  </si>
+  <si>
+    <t>+4.1%</t>
+  </si>
+  <si>
+    <t>Professional Services</t>
+  </si>
+  <si>
+    <t>190,000</t>
+  </si>
+  <si>
+    <t>210,000</t>
+  </si>
+  <si>
+    <t>230,000</t>
+  </si>
+  <si>
+    <t>+9.5%</t>
+  </si>
+  <si>
+    <t>Total Net Revenue</t>
+  </si>
+  <si>
+    <t>1,770,500</t>
+  </si>
+  <si>
+    <t>2,055,200</t>
+  </si>
+  <si>
+    <t>2,260,000</t>
+  </si>
+  <si>
+    <t>+10.0%</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Budget Allocation</t>
+  </si>
+  <si>
+    <t>Spent to Date</t>
+  </si>
+  <si>
+    <t>Remaining Balance</t>
+  </si>
+  <si>
+    <t>R&amp;D Core Engineering</t>
+  </si>
+  <si>
+    <t>850,000</t>
+  </si>
+  <si>
+    <t>590,000</t>
+  </si>
+  <si>
+    <t>260,000</t>
+  </si>
+  <si>
+    <t>Product Design</t>
+  </si>
+  <si>
+    <t>220,000</t>
+  </si>
+  <si>
+    <t>145,000</t>
+  </si>
+  <si>
+    <t>75,000</t>
+  </si>
+  <si>
+    <t>Quality Assurance</t>
+  </si>
+  <si>
+    <t>160,000</t>
+  </si>
+  <si>
+    <t>110,000</t>
+  </si>
+  <si>
+    <t>50,000</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>